<commit_message>
Audited corpus: 40 CORE (10 records reclassified to EXCLUDE); regenerate screening flow, PRISMA and tests
</commit_message>
<xml_diff>
--- a/data/screening/manual_screening.xlsx
+++ b/data/screening/manual_screening.xlsx
@@ -749,7 +749,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2604.21210</t>
+          <t>2602.03405</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr"/>
@@ -760,7 +760,7 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>The Feedback Hamiltonian is the Score Function: A Diffusion-Model Framework for Quantum Trajectory Reversal</t>
+          <t>Enhancing Quantum Diffusion Models for Complex Image Generation</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -775,20 +775,20 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr"/>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>Feedback Hamiltonian as score function; diffusion-model framework for quantum.</t>
+          <t>Hybrid Q-C U-Net QDM for complex images.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>2602.03405</t>
+          <t>2605.01367</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr"/>
@@ -799,7 +799,7 @@
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>Enhancing Quantum Diffusion Models for Complex Image Generation</t>
+          <t>From Characterization To Construction: Generative Quantum Circuit Synthesis from Gate Set Tomography Data</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
@@ -820,14 +820,14 @@
       <c r="H7" s="3" t="inlineStr"/>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>Hybrid Q-C U-Net QDM for complex images.</t>
+          <t>Generative quantum circuit synthesis from gate sets.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2605.01367</t>
+          <t>2606.29636</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr"/>
@@ -838,7 +838,7 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>From Characterization To Construction: Generative Quantum Circuit Synthesis from Gate Set Tomography Data</t>
+          <t>Lie Group Diffusion Models for Hardware-Aware Quantum Circuit Synthesis</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -859,17 +859,21 @@
       <c r="H8" s="3" t="inlineStr"/>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>Generative quantum circuit synthesis from gate sets.</t>
+          <t>Lie-group diffusion models for hardware-aware circuit synthesis.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>2606.29636</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr"/>
+          <t>2509.14163</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>10.1109/icassp55912.2026.11461991</t>
+        </is>
+      </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
           <t>2026</t>
@@ -877,7 +881,7 @@
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>Lie Group Diffusion Models for Hardware-Aware Quantum Circuit Synthesis</t>
+          <t>Quantum Reinforcement Learning-Guided Diffusion Model for Image Synthesis via Hybrid Quantum-Classical Generative Model Architectures</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -892,23 +896,27 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="H9" s="3" t="inlineStr"/>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>Lie-group diffusion models for hardware-aware circuit synthesis.</t>
+          <t>Quantum RL-guided hybrid diffusion for image synthesis.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2605.23403</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr"/>
+          <t>2509.17324</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>10.1109/icassp55912.2026.11461326</t>
+        </is>
+      </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
           <t>2026</t>
@@ -916,7 +924,7 @@
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>Hybrid Quantum-Classical Corrective Diffusion Modeling for Meteorological Downscaling</t>
+          <t>DiffQ: Unified Parameter Initialization for Variational Quantum Algorithms Via Diffusion Models</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -937,17 +945,21 @@
       <c r="H10" s="3" t="inlineStr"/>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>Hybrid quantum-classical corrective diffusion (meteorological downscaling).</t>
+          <t>DiffQ: diffusion for VQA parameter initialization (circuit-adjacent).</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>2606.05217</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr"/>
+          <t>2512.20448</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>10.1109/tgrs.2026.3661445</t>
+        </is>
+      </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
           <t>2026</t>
@@ -955,7 +967,7 @@
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>The Score Hamiltonian: Mapping Diffusion Models to Adiabatic Transport</t>
+          <t>Enriching Earth Observation Labeled Data With Quantum Conditioned Diffusion Models</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
@@ -970,25 +982,21 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="H11" s="3" t="inlineStr"/>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>Theory: mapping diffusion models to adiabatic transport (Score Hamiltonian).</t>
+          <t>Quantum conditioned diffusion for Earth-observation data.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>2509.14163</t>
-        </is>
-      </c>
+      <c r="A12" s="2" t="inlineStr"/>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>10.1109/icassp55912.2026.11461991</t>
+          <t>10.1007/s42484-026-00352-1</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -998,7 +1006,7 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>Quantum Reinforcement Learning-Guided Diffusion Model for Image Synthesis via Hybrid Quantum-Classical Generative Model Architectures</t>
+          <t>Quantum latent diffusion model for high-dimensional state generation</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
@@ -1013,27 +1021,23 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="H12" s="3" t="inlineStr"/>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>Quantum RL-guided hybrid diffusion for image synthesis.</t>
+          <t>Quantum latent diffusion for high-dimensional state generation (QMI).</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>2509.17324</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>10.1109/icassp55912.2026.11461326</t>
-        </is>
-      </c>
+          <t>2603.06488</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr"/>
       <c r="C13" s="2" t="inlineStr">
         <is>
           <t>2026</t>
@@ -1041,7 +1045,7 @@
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>DiffQ: Unified Parameter Initialization for Variational Quantum Algorithms Via Diffusion Models</t>
+          <t>Score Reversal Is Not Free for Quantum Diffusion Models</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
@@ -1056,25 +1060,21 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="H13" s="3" t="inlineStr"/>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>DiffQ: diffusion for VQA parameter initialization (circuit-adjacent).</t>
+          <t>No-go theory for reverse quantum diffusion.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>2512.20448</t>
-        </is>
-      </c>
+      <c r="A14" s="2" t="inlineStr"/>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>10.1109/tgrs.2026.3661445</t>
+          <t>10.1007/978-3-032-15931-1_4</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -1084,12 +1084,12 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>Enriching Earth Observation Labeled Data With Quantum Conditioned Diffusion Models</t>
+          <t>Quantum Diffusion Models for Few-Shot Learning</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>CORE</t>
+          <t>MANUAL_REVIEW</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
@@ -1099,31 +1099,31 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="H14" s="3" t="inlineStr"/>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>Quantum conditioned diffusion for Earth-observation data.</t>
+          <t>QDM for few-shot learning (book chapter; possible duplicate of 2411.04217).</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="inlineStr"/>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>10.1007/s42484-026-00352-1</t>
-        </is>
-      </c>
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>2512.06695</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr"/>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>Quantum latent diffusion model for high-dimensional state generation</t>
+          <t>Mitigating Barren Plateaus in Quantum Denoising Diffusion Probabilistic Model</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
@@ -1144,25 +1144,25 @@
       <c r="H15" s="3" t="inlineStr"/>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>Quantum latent diffusion for high-dimensional state generation (QMI).</t>
+          <t>QuDDPM barren-plateau mitigation.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2603.06488</t>
+          <t>2505.05151</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr"/>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>Score Reversal Is Not Free for Quantum Diffusion Models</t>
+          <t>Overcoming Dimensional Factorization Limits in Discrete Diffusion Models through Quantum Joint Distribution Learning</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
@@ -1183,30 +1183,30 @@
       <c r="H16" s="3" t="inlineStr"/>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>No-go theory for reverse quantum diffusion.</t>
+          <t>Quantum discrete diffusion (dimensional factorization limits).</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="inlineStr"/>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>10.1007/978-3-032-15931-1_4</t>
-        </is>
-      </c>
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>2509.17569</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr"/>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>Quantum Diffusion Models for Few-Shot Learning</t>
+          <t>Conditioning in Generative Quantum Denoising Diffusion Models</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>MANUAL_REVIEW</t>
+          <t>CORE</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
@@ -1216,23 +1216,27 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="H17" s="3" t="inlineStr"/>
       <c r="I17" s="3" t="inlineStr">
         <is>
-          <t>QDM for few-shot learning (book chapter; possible duplicate of 2411.04217).</t>
+          <t>Conditioning in generative QuDDPM.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2512.06695</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr"/>
+          <t>2506.01666</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>10.1088/2632-2153/ae5b21</t>
+        </is>
+      </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
           <t>2025</t>
@@ -1240,7 +1244,7 @@
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>Mitigating Barren Plateaus in Quantum Denoising Diffusion Probabilistic Model</t>
+          <t>Synthesis of discrete-continuous quantum circuits with multimodal diffusion models</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
@@ -1261,14 +1265,14 @@
       <c r="H18" s="3" t="inlineStr"/>
       <c r="I18" s="3" t="inlineStr">
         <is>
-          <t>QuDDPM barren-plateau mitigation.</t>
+          <t>Multimodal diffusion for discrete-continuous circuit synthesis.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>2505.05151</t>
+          <t>2506.19270</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr"/>
@@ -1279,7 +1283,7 @@
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>Overcoming Dimensional Factorization Limits in Discrete Diffusion Models through Quantum Joint Distribution Learning</t>
+          <t>Continuous-variable Quantum Diffusion Model for State Generation and Restoration</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
@@ -1300,14 +1304,14 @@
       <c r="H19" s="3" t="inlineStr"/>
       <c r="I19" s="3" t="inlineStr">
         <is>
-          <t>Quantum discrete diffusion (dimensional factorization limits).</t>
+          <t>Continuous-variable quantum diffusion model.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2501.05666</t>
+          <t>2501.16380</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr"/>
@@ -1318,7 +1322,7 @@
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>Diffusion-Enhanced Optimization of Variational Quantum Eigensolver for General Hamiltonians</t>
+          <t>UDiTQC: U-Net-Style Diffusion Transformer for Quantum Circuit Synthesis</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
@@ -1333,20 +1337,20 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="H20" s="3" t="inlineStr"/>
       <c r="I20" s="3" t="inlineStr">
         <is>
-          <t>Diffusion-enhanced VQE optimization (diffusion for quantum optimization).</t>
+          <t>U-Net diffusion transformer for quantum circuit synthesis.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>2509.17569</t>
+          <t>2505.22193</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr"/>
@@ -1357,7 +1361,7 @@
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>Conditioning in Generative Quantum Denoising Diffusion Models</t>
+          <t>Physics-inspired Generative AI models via real hardware-based noisy quantum diffusion</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
@@ -1378,21 +1382,17 @@
       <c r="H21" s="3" t="inlineStr"/>
       <c r="I21" s="3" t="inlineStr">
         <is>
-          <t>Conditioning in generative QuDDPM.</t>
+          <t>Noise-driven QDM on real hardware.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2506.01666</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>10.1088/2632-2153/ae5b21</t>
-        </is>
-      </c>
+          <t>2508.08799</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr"/>
       <c r="C22" s="2" t="inlineStr">
         <is>
           <t>2025</t>
@@ -1400,7 +1400,7 @@
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>Synthesis of discrete-continuous quantum circuits with multimodal diffusion models</t>
+          <t>Measurement-Based Quantum Diffusion Models</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
@@ -1421,17 +1421,21 @@
       <c r="H22" s="3" t="inlineStr"/>
       <c r="I22" s="3" t="inlineStr">
         <is>
-          <t>Multimodal diffusion for discrete-continuous circuit synthesis.</t>
+          <t>Measurement-based quantum diffusion.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>2506.19270</t>
-        </is>
-      </c>
-      <c r="B23" s="2" t="inlineStr"/>
+          <t>2505.20863</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>10.1109/qce65121.2025.00180</t>
+        </is>
+      </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
           <t>2025</t>
@@ -1439,7 +1443,7 @@
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>Continuous-variable Quantum Diffusion Model for State Generation and Restoration</t>
+          <t>Leveraging Diffusion Models for Parameterized Quantum Circuit Generation</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
@@ -1460,14 +1464,14 @@
       <c r="H23" s="3" t="inlineStr"/>
       <c r="I23" s="3" t="inlineStr">
         <is>
-          <t>Continuous-variable quantum diffusion model.</t>
+          <t>Diffusion for parameterized quantum circuit generation (Barta).</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2501.16380</t>
+          <t>2511.12221</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr"/>
@@ -1478,7 +1482,7 @@
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>UDiTQC: U-Net-Style Diffusion Transformer for Quantum Circuit Synthesis</t>
+          <t>Channel-Constrained Markovian Quantum Diffusion Model from Open System Perspective</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
@@ -1499,17 +1503,21 @@
       <c r="H24" s="3" t="inlineStr"/>
       <c r="I24" s="3" t="inlineStr">
         <is>
-          <t>U-Net diffusion transformer for quantum circuit synthesis.</t>
+          <t>Open-system Markovian quantum diffusion (CCMQD).</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>2505.22193</t>
-        </is>
-      </c>
-      <c r="B25" s="2" t="inlineStr"/>
+          <t>2411.15973</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>10.1007/978-3-031-78395-1_23</t>
+        </is>
+      </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
           <t>2025</t>
@@ -1517,7 +1525,7 @@
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>Physics-inspired Generative AI models via real hardware-based noisy quantum diffusion</t>
+          <t>Enhancing Quantum Diffusion Models with Pairwise Bell State Entanglement</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
@@ -1538,17 +1546,21 @@
       <c r="H25" s="3" t="inlineStr"/>
       <c r="I25" s="3" t="inlineStr">
         <is>
-          <t>Noise-driven QDM on real hardware.</t>
+          <t>Bell-state entanglement QDM.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2508.08799</t>
-        </is>
-      </c>
-      <c r="B26" s="2" t="inlineStr"/>
+          <t>2508.09903</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>10.1109/qce65121.2025.10364</t>
+        </is>
+      </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
           <t>2025</t>
@@ -1556,7 +1568,7 @@
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>Measurement-Based Quantum Diffusion Models</t>
+          <t>Hybrid Quantum-Classical Latent Diffusion Models for Medical Image Generation</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
@@ -1577,19 +1589,19 @@
       <c r="H26" s="3" t="inlineStr"/>
       <c r="I26" s="3" t="inlineStr">
         <is>
-          <t>Measurement-based quantum diffusion.</t>
+          <t>Hybrid latent QDM for medical imaging.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>2505.20863</t>
+          <t>2411.04217</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>10.1109/qce65121.2025.00180</t>
+          <t>10.1109/icad65464.2025.11114033</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
@@ -1599,7 +1611,7 @@
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>Leveraging Diffusion Models for Parameterized Quantum Circuit Generation</t>
+          <t>Quantum Diffusion Models for Few-Shot Learning</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
@@ -1620,17 +1632,21 @@
       <c r="H27" s="3" t="inlineStr"/>
       <c r="I27" s="3" t="inlineStr">
         <is>
-          <t>Diffusion for parameterized quantum circuit generation (Barta).</t>
+          <t>QDM for few-shot learning.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2511.12221</t>
-        </is>
-      </c>
-      <c r="B28" s="2" t="inlineStr"/>
+          <t>2406.00843</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>10.1007/s42484-025-00276-2</t>
+        </is>
+      </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
           <t>2025</t>
@@ -1638,7 +1654,7 @@
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>Channel-Constrained Markovian Quantum Diffusion Model from Open System Perspective</t>
+          <t>Diffusion-inspired quantum noise mitigation in parameterized quantum circuits</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
@@ -1653,25 +1669,25 @@
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="H28" s="3" t="inlineStr"/>
       <c r="I28" s="3" t="inlineStr">
         <is>
-          <t>Open-system Markovian quantum diffusion (CCMQD).</t>
+          <t>Diffusion-inspired quantum noise mitigation in PQCs (QMI).</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>2411.15973</t>
+          <t>2501.11174</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>10.1007/978-3-031-78395-1_23</t>
+          <t>10.1007/s42484-024-00224-6</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
@@ -1681,12 +1697,12 @@
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>Enhancing Quantum Diffusion Models with Pairwise Bell State Entanglement</t>
+          <t>Quantum Latent Diffusion Models</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>CORE</t>
+          <t>MANUAL_REVIEW</t>
         </is>
       </c>
       <c r="F29" s="4" t="inlineStr">
@@ -1702,19 +1718,15 @@
       <c r="H29" s="3" t="inlineStr"/>
       <c r="I29" s="3" t="inlineStr">
         <is>
-          <t>Bell-state entanglement QDM.</t>
+          <t>Quantum Latent Diffusion Models (De Falco, QMI).</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="2" t="inlineStr">
-        <is>
-          <t>2508.09903</t>
-        </is>
-      </c>
+      <c r="A30" s="2" t="inlineStr"/>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>10.1109/qce65121.2025.10364</t>
+          <t>10.1109/ijcnn64981.2025.11227283</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
@@ -1724,12 +1736,12 @@
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>Hybrid Quantum-Classical Latent Diffusion Models for Medical Image Generation</t>
+          <t>Hybrid and hardware-oriented approaches for quantum diffusion models</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>CORE</t>
+          <t>MANUAL_REVIEW</t>
         </is>
       </c>
       <c r="F30" s="4" t="inlineStr">
@@ -1745,19 +1757,15 @@
       <c r="H30" s="3" t="inlineStr"/>
       <c r="I30" s="3" t="inlineStr">
         <is>
-          <t>Hybrid latent QDM for medical imaging.</t>
+          <t>Hybrid hardware-oriented quantum diffusion approaches.</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="2" t="inlineStr">
-        <is>
-          <t>2411.04217</t>
-        </is>
-      </c>
+      <c r="A31" s="2" t="inlineStr"/>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>10.1109/icad65464.2025.11114033</t>
+          <t>10.1109/igarss55030.2025.11242723</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
@@ -1767,12 +1775,12 @@
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>Quantum Diffusion Models for Few-Shot Learning</t>
+          <t>Leveraging Quantum Latent Diffusion Models for Data Augmentation on The Eurosat Dataset</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>CORE</t>
+          <t>MANUAL_REVIEW</t>
         </is>
       </c>
       <c r="F31" s="4" t="inlineStr">
@@ -1788,29 +1796,25 @@
       <c r="H31" s="3" t="inlineStr"/>
       <c r="I31" s="3" t="inlineStr">
         <is>
-          <t>QDM for few-shot learning.</t>
+          <t>Quantum latent diffusion for EuroSAT data augmentation.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2406.00843</t>
-        </is>
-      </c>
-      <c r="B32" s="2" t="inlineStr">
-        <is>
-          <t>10.1007/s42484-025-00276-2</t>
-        </is>
-      </c>
+          <t>2411.17608</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr"/>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>Diffusion-inspired quantum noise mitigation in parameterized quantum circuits</t>
+          <t>Mixed-State Quantum Denoising Diffusion Probabilistic Model</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
@@ -1825,40 +1829,36 @@
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="H32" s="3" t="inlineStr"/>
       <c r="I32" s="3" t="inlineStr">
         <is>
-          <t>Diffusion-inspired quantum noise mitigation in PQCs (QMI).</t>
+          <t>Mixed-state QuDDPM (Kwun).</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>2501.11174</t>
-        </is>
-      </c>
-      <c r="B33" s="2" t="inlineStr">
-        <is>
-          <t>10.1007/s42484-024-00224-6</t>
-        </is>
-      </c>
+          <t>2407.12242</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr"/>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>Quantum Latent Diffusion Models</t>
+          <t>Conditional Diffusion-based Parameter Generation for Quantum Approximate Optimization Algorithm</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>MANUAL_REVIEW</t>
+          <t>CORE</t>
         </is>
       </c>
       <c r="F33" s="4" t="inlineStr">
@@ -1874,30 +1874,34 @@
       <c r="H33" s="3" t="inlineStr"/>
       <c r="I33" s="3" t="inlineStr">
         <is>
-          <t>Quantum Latent Diffusion Models (De Falco, QMI).</t>
+          <t>Conditional diffusion for QAOA parameter generation.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2512.19877</t>
-        </is>
-      </c>
-      <c r="B34" s="2" t="inlineStr"/>
+          <t>2401.07049</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>10.1109/qsw62656.2024.00023</t>
+        </is>
+      </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>Spectral Diffusion for Sampling on ${\rm SU}(N)$</t>
+          <t>Quantum Denoising Diffusion Models</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>MANUAL_REVIEW</t>
+          <t>CORE</t>
         </is>
       </c>
       <c r="F34" s="4" t="inlineStr">
@@ -1907,36 +1911,36 @@
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="H34" s="3" t="inlineStr"/>
       <c r="I34" s="3" t="inlineStr">
         <is>
-          <t>Spectral diffusion for sampling on SU(N).</t>
+          <t>Quantum Denoising Diffusion Models (Kolle).</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="2" t="inlineStr"/>
-      <c r="B35" s="2" t="inlineStr">
-        <is>
-          <t>10.1109/ijcnn64981.2025.11227283</t>
-        </is>
-      </c>
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>2412.21082</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr"/>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>Hybrid and hardware-oriented approaches for quantum diffusion models</t>
+          <t>Quantum Diffusion Model for Quark and Gluon Jet Generation</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>MANUAL_REVIEW</t>
+          <t>CORE</t>
         </is>
       </c>
       <c r="F35" s="4" t="inlineStr">
@@ -1952,30 +1956,34 @@
       <c r="H35" s="3" t="inlineStr"/>
       <c r="I35" s="3" t="inlineStr">
         <is>
-          <t>Hybrid hardware-oriented quantum diffusion approaches.</t>
+          <t>QDM for quark/gluon jet generation.</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="2" t="inlineStr"/>
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>2402.16147</t>
+        </is>
+      </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>10.1109/igarss55030.2025.11242723</t>
+          <t>10.1007/s13218-024-00858-5</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>Leveraging Quantum Latent Diffusion Models for Data Augmentation on The Eurosat Dataset</t>
+          <t>Towards Efficient Quantum Hybrid Diffusion Models</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>MANUAL_REVIEW</t>
+          <t>CORE</t>
         </is>
       </c>
       <c r="F36" s="4" t="inlineStr">
@@ -1991,17 +1999,17 @@
       <c r="H36" s="3" t="inlineStr"/>
       <c r="I36" s="3" t="inlineStr">
         <is>
-          <t>Quantum latent diffusion for EuroSAT data augmentation.</t>
+          <t>Towards efficient quantum hybrid diffusion (De Falco).</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="2" t="inlineStr">
-        <is>
-          <t>2411.17608</t>
-        </is>
-      </c>
-      <c r="B37" s="2" t="inlineStr"/>
+      <c r="A37" s="2" t="inlineStr"/>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>10.1109/qce60285.2024.10371</t>
+        </is>
+      </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
           <t>2024</t>
@@ -2009,12 +2017,12 @@
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>Mixed-State Quantum Denoising Diffusion Probabilistic Model</t>
+          <t>Understanding of the Diffusion Noise in Quantum Latent Diffusion Model</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>CORE</t>
+          <t>MANUAL_REVIEW</t>
         </is>
       </c>
       <c r="F37" s="4" t="inlineStr">
@@ -2024,31 +2032,35 @@
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="H37" s="3" t="inlineStr"/>
       <c r="I37" s="3" t="inlineStr">
         <is>
-          <t>Mixed-state QuDDPM (Kwun).</t>
+          <t>Analysis of diffusion noise in quantum latent diffusion.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2407.12242</t>
-        </is>
-      </c>
-      <c r="B38" s="2" t="inlineStr"/>
+          <t>2311.02041</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>10.1038/s42256-024-00831-9</t>
+        </is>
+      </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2023</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>Conditional Diffusion-based Parameter Generation for Quantum Approximate Optimization Algorithm</t>
+          <t>Quantum circuit synthesis with diffusion models</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
@@ -2069,29 +2081,25 @@
       <c r="H38" s="3" t="inlineStr"/>
       <c r="I38" s="3" t="inlineStr">
         <is>
-          <t>Conditional diffusion for QAOA parameter generation.</t>
+          <t>Quantum circuit synthesis with diffusion (genQC, Furrutter).</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>2401.07049</t>
-        </is>
-      </c>
-      <c r="B39" s="2" t="inlineStr">
-        <is>
-          <t>10.1109/qsw62656.2024.00023</t>
-        </is>
-      </c>
+          <t>2310.02511</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr"/>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2023</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
         <is>
-          <t>Quantum Denoising Diffusion Models</t>
+          <t>Prepare Ansatz for VQE with Diffusion Model</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
@@ -2112,25 +2120,25 @@
       <c r="H39" s="3" t="inlineStr"/>
       <c r="I39" s="3" t="inlineStr">
         <is>
-          <t>Quantum Denoising Diffusion Models (Kolle).</t>
+          <t>Diffusion model to prepare VQE ansatz.</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="2" t="inlineStr"/>
-      <c r="B40" s="2" t="inlineStr">
-        <is>
-          <t>10.1109/qce60285.2024.10259</t>
-        </is>
-      </c>
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>2311.15444</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr"/>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2023</t>
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>QRNG-DDPM: Enhancing Diffusion Models Through Fitting Mixture Noise with Quantum Random Number</t>
+          <t>Quantum Diffusion Models</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
@@ -2145,36 +2153,40 @@
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="H40" s="3" t="inlineStr"/>
       <c r="I40" s="3" t="inlineStr">
         <is>
-          <t>QRNG-DDPM: quantum random noise in DDPM (hybrid quantum component).</t>
+          <t>Quantum Diffusion Models (Cacioppo).</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>2412.21082</t>
-        </is>
-      </c>
-      <c r="B41" s="2" t="inlineStr"/>
+          <t>2310.05866</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>10.1103/physrevlett.132.100602</t>
+        </is>
+      </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2023</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>Quantum Diffusion Model for Quark and Gluon Jet Generation</t>
+          <t>Generative quantum machine learning via denoising diffusion probabilistic models</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>CORE</t>
+          <t>MANUAL_REVIEW</t>
         </is>
       </c>
       <c r="F41" s="4" t="inlineStr">
@@ -2190,29 +2202,25 @@
       <c r="H41" s="3" t="inlineStr"/>
       <c r="I41" s="3" t="inlineStr">
         <is>
-          <t>QDM for quark/gluon jet generation.</t>
+          <t>Generative QML via DDPM (Zhang QuDDPM; foundational).</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2402.16147</t>
-        </is>
-      </c>
-      <c r="B42" s="2" t="inlineStr">
-        <is>
-          <t>10.1007/s13218-024-00858-5</t>
-        </is>
-      </c>
+          <t>2601.22005</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr"/>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t>Towards Efficient Quantum Hybrid Diffusion Models</t>
+          <t>Hierarchy of discriminative power and complexity in learning quantum ensembles</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
@@ -2220,9 +2228,9 @@
           <t>CORE</t>
         </is>
       </c>
-      <c r="F42" s="4" t="inlineStr">
-        <is>
-          <t>CORE</t>
+      <c r="F42" s="5" t="inlineStr">
+        <is>
+          <t>RELATED</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
@@ -2233,35 +2241,35 @@
       <c r="H42" s="3" t="inlineStr"/>
       <c r="I42" s="3" t="inlineStr">
         <is>
-          <t>Towards efficient quantum hybrid diffusion (De Falco).</t>
+          <t>MMD-k evaluation metric for quantum ensembles; supporting, not a generative model.</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="2" t="inlineStr"/>
-      <c r="B43" s="2" t="inlineStr">
-        <is>
-          <t>10.1109/tpami.2024.3430839</t>
-        </is>
-      </c>
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>2606.28483</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr"/>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr">
         <is>
-          <t>STQD-Det: Spatio-Temporal Quantum Diffusion Model for Real-Time Coronary Stenosis Detection in X-Ray Angiography</t>
+          <t>Quantum Fourier Generative Models Trainable at Large Scale</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="F43" s="6" t="inlineStr">
+        <is>
           <t>MANUAL_REVIEW</t>
-        </is>
-      </c>
-      <c r="F43" s="4" t="inlineStr">
-        <is>
-          <t>CORE</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
@@ -2272,35 +2280,35 @@
       <c r="H43" s="3" t="inlineStr"/>
       <c r="I43" s="3" t="inlineStr">
         <is>
-          <t>Spatio-temporal quantum diffusion for stenosis detection (STQD-Det).</t>
+          <t>Quantum Fourier generative models; unclear if diffusion-based. Needs full text.</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="2" t="inlineStr"/>
-      <c r="B44" s="2" t="inlineStr">
-        <is>
-          <t>10.1109/qce60285.2024.10371</t>
-        </is>
-      </c>
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>2604.01197</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr"/>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>Understanding of the Diffusion Noise in Quantum Latent Diffusion Model</t>
+          <t>Learning and Generating Mixed States Prepared by Shallow Channel Circuits</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="F44" s="6" t="inlineStr">
+        <is>
           <t>MANUAL_REVIEW</t>
-        </is>
-      </c>
-      <c r="F44" s="4" t="inlineStr">
-        <is>
-          <t>CORE</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
@@ -2311,21 +2319,17 @@
       <c r="H44" s="3" t="inlineStr"/>
       <c r="I44" s="3" t="inlineStr">
         <is>
-          <t>Analysis of diffusion noise in quantum latent diffusion.</t>
+          <t>Generating mixed states via shallow channels; verify it is diffusion-based.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>2311.02041</t>
-        </is>
-      </c>
-      <c r="B45" s="2" t="inlineStr">
-        <is>
-          <t>10.1038/s42256-024-00831-9</t>
-        </is>
-      </c>
+          <t>2310.07797</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr"/>
       <c r="C45" s="2" t="inlineStr">
         <is>
           <t>2023</t>
@@ -2333,7 +2337,7 @@
       </c>
       <c r="D45" s="3" t="inlineStr">
         <is>
-          <t>Quantum circuit synthesis with diffusion models</t>
+          <t>Quantum sequential scattering model for quantum state learning</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
@@ -2341,38 +2345,42 @@
           <t>CORE</t>
         </is>
       </c>
-      <c r="F45" s="4" t="inlineStr">
-        <is>
-          <t>CORE</t>
+      <c r="F45" s="6" t="inlineStr">
+        <is>
+          <t>MANUAL_REVIEW</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="H45" s="3" t="inlineStr"/>
       <c r="I45" s="3" t="inlineStr">
         <is>
-          <t>Quantum circuit synthesis with diffusion (genQC, Furrutter).</t>
+          <t>Quantum sequential scattering for state learning; verify diffusion link.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2310.02511</t>
-        </is>
-      </c>
-      <c r="B46" s="2" t="inlineStr"/>
+          <t>2603.02834</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>10.15302/frontphys.2026.113201</t>
+        </is>
+      </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t>Prepare Ansatz for VQE with Diffusion Model</t>
+          <t>Identification of quantum generative circuits with parallel quantum neural network</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
@@ -2380,9 +2388,9 @@
           <t>CORE</t>
         </is>
       </c>
-      <c r="F46" s="4" t="inlineStr">
-        <is>
-          <t>CORE</t>
+      <c r="F46" s="7" t="inlineStr">
+        <is>
+          <t>EXCLUDE</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
@@ -2390,28 +2398,32 @@
           <t>high</t>
         </is>
       </c>
-      <c r="H46" s="3" t="inlineStr"/>
+      <c r="H46" s="3" t="inlineStr">
+        <is>
+          <t>Discriminative circuit identification (ParaQuanNet); not generative diffusion.</t>
+        </is>
+      </c>
       <c r="I46" s="3" t="inlineStr">
         <is>
-          <t>Diffusion model to prepare VQE ansatz.</t>
+          <t>Discriminative circuit identification (ParaQuanNet); not generative diffusion.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>2305.16540</t>
+          <t>2604.21210</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr"/>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t>A Score-Based Model for Learning Neural Wavefunctions</t>
+          <t>The Feedback Hamiltonian is the Score Function: A Diffusion-Model Framework for Quantum Trajectory Reversal</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
@@ -2419,38 +2431,42 @@
           <t>CORE</t>
         </is>
       </c>
-      <c r="F47" s="4" t="inlineStr">
-        <is>
-          <t>CORE</t>
+      <c r="F47" s="7" t="inlineStr">
+        <is>
+          <t>EXCLUDE</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="H47" s="3" t="inlineStr"/>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="H47" s="3" t="inlineStr">
+        <is>
+          <t>Removed in manual audit: insufficient relation to quantum diffusion models.</t>
+        </is>
+      </c>
       <c r="I47" s="3" t="inlineStr">
         <is>
-          <t>Score-based model for learning neural wavefunctions.</t>
+          <t>Reclassified from CORE/RELATED to EXCLUDE during manual audit (2026-07-13).</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2311.15444</t>
+          <t>2605.19754</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr"/>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>Quantum Diffusion Models</t>
+          <t>Hypothesis Tests for Observing Quantum Entanglement in HWW at the LHC</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
@@ -2458,9 +2474,9 @@
           <t>CORE</t>
         </is>
       </c>
-      <c r="F48" s="4" t="inlineStr">
-        <is>
-          <t>CORE</t>
+      <c r="F48" s="7" t="inlineStr">
+        <is>
+          <t>EXCLUDE</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
@@ -2468,42 +2484,42 @@
           <t>high</t>
         </is>
       </c>
-      <c r="H48" s="3" t="inlineStr"/>
+      <c r="H48" s="3" t="inlineStr">
+        <is>
+          <t>LHC particle-physics entanglement hypothesis test; off-topic.</t>
+        </is>
+      </c>
       <c r="I48" s="3" t="inlineStr">
         <is>
-          <t>Quantum Diffusion Models (Cacioppo).</t>
+          <t>LHC particle-physics entanglement hypothesis test; off-topic.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>2310.05866</t>
-        </is>
-      </c>
-      <c r="B49" s="2" t="inlineStr">
-        <is>
-          <t>10.1103/physrevlett.132.100602</t>
-        </is>
-      </c>
+          <t>2605.23403</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr"/>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="D49" s="3" t="inlineStr">
         <is>
-          <t>Generative quantum machine learning via denoising diffusion probabilistic models</t>
+          <t>Hybrid Quantum-Classical Corrective Diffusion Modeling for Meteorological Downscaling</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>MANUAL_REVIEW</t>
-        </is>
-      </c>
-      <c r="F49" s="4" t="inlineStr">
-        <is>
-          <t>CORE</t>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="F49" s="7" t="inlineStr">
+        <is>
+          <t>EXCLUDE</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
@@ -2511,17 +2527,21 @@
           <t>high</t>
         </is>
       </c>
-      <c r="H49" s="3" t="inlineStr"/>
+      <c r="H49" s="3" t="inlineStr">
+        <is>
+          <t>Removed in manual audit: insufficient relation to quantum diffusion models.</t>
+        </is>
+      </c>
       <c r="I49" s="3" t="inlineStr">
         <is>
-          <t>Generative QML via DDPM (Zhang QuDDPM; foundational).</t>
+          <t>Reclassified from CORE/RELATED to EXCLUDE during manual audit (2026-07-13).</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2601.22005</t>
+          <t>2606.05217</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr"/>
@@ -2532,7 +2552,7 @@
       </c>
       <c r="D50" s="3" t="inlineStr">
         <is>
-          <t>Hierarchy of discriminative power and complexity in learning quantum ensembles</t>
+          <t>The Score Hamiltonian: Mapping Diffusion Models to Adiabatic Transport</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
@@ -2540,9 +2560,9 @@
           <t>CORE</t>
         </is>
       </c>
-      <c r="F50" s="5" t="inlineStr">
-        <is>
-          <t>RELATED</t>
+      <c r="F50" s="7" t="inlineStr">
+        <is>
+          <t>EXCLUDE</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
@@ -2550,17 +2570,21 @@
           <t>high</t>
         </is>
       </c>
-      <c r="H50" s="3" t="inlineStr"/>
+      <c r="H50" s="3" t="inlineStr">
+        <is>
+          <t>Removed in manual audit: insufficient relation to quantum diffusion models.</t>
+        </is>
+      </c>
       <c r="I50" s="3" t="inlineStr">
         <is>
-          <t>MMD-k evaluation metric for quantum ensembles; supporting, not a generative model.</t>
+          <t>Reclassified from CORE/RELATED to EXCLUDE during manual audit (2026-07-13).</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>2605.13268</t>
+          <t>2607.00566</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr"/>
@@ -2571,46 +2595,50 @@
       </c>
       <c r="D51" s="3" t="inlineStr">
         <is>
-          <t>Physics Guided Generative Optimization for Trotter Suzuki Decomposition</t>
+          <t>Effective Color Dipole Approach to Color Transparency in $ρ^0$ Electroproduction</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>RELATED</t>
-        </is>
-      </c>
-      <c r="F51" s="5" t="inlineStr">
-        <is>
-          <t>RELATED</t>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="F51" s="7" t="inlineStr">
+        <is>
+          <t>EXCLUDE</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="H51" s="3" t="inlineStr"/>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="H51" s="3" t="inlineStr">
+        <is>
+          <t>Nuclear-physics color transparency; transport, not generative.</t>
+        </is>
+      </c>
       <c r="I51" s="3" t="inlineStr">
         <is>
-          <t>Generative optimization for Trotter-Suzuki decomposition; not diffusion.</t>
+          <t>Nuclear-physics color transparency; transport, not generative.</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="2" t="inlineStr"/>
-      <c r="B52" s="2" t="inlineStr">
-        <is>
-          <t>10.1007/jhep05(2024)060</t>
-        </is>
-      </c>
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>2604.05612</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr"/>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="D52" s="3" t="inlineStr">
         <is>
-          <t>Diffusion models as stochastic quantization in lattice field theory</t>
+          <t>Deuteron normalization and channel-dependent formation dynamics in pion and kaon color transparency</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
@@ -2618,30 +2646,34 @@
           <t>MANUAL_REVIEW</t>
         </is>
       </c>
-      <c r="F52" s="5" t="inlineStr">
-        <is>
-          <t>RELATED</t>
+      <c r="F52" s="7" t="inlineStr">
+        <is>
+          <t>EXCLUDE</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="H52" s="3" t="inlineStr"/>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="H52" s="3" t="inlineStr">
+        <is>
+          <t>Nuclear-physics color transparency; off-topic.</t>
+        </is>
+      </c>
       <c r="I52" s="3" t="inlineStr">
         <is>
-          <t>Diffusion models as stochastic quantization in lattice field theory; conceptual link.</t>
+          <t>Nuclear-physics color transparency; off-topic.</t>
         </is>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="2" t="inlineStr">
-        <is>
-          <t>2606.28483</t>
-        </is>
-      </c>
-      <c r="B53" s="2" t="inlineStr"/>
+      <c r="A53" s="2" t="inlineStr"/>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>10.1007/978-3-032-09973-0_7</t>
+        </is>
+      </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
           <t>2026</t>
@@ -2649,35 +2681,39 @@
       </c>
       <c r="D53" s="3" t="inlineStr">
         <is>
-          <t>Quantum Fourier Generative Models Trainable at Large Scale</t>
+          <t>Ecological Pollution Control Using a Nonlinear Diffusion Model Based on Quantum Optimization</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>CORE</t>
-        </is>
-      </c>
-      <c r="F53" s="6" t="inlineStr">
-        <is>
           <t>MANUAL_REVIEW</t>
         </is>
       </c>
+      <c r="F53" s="7" t="inlineStr">
+        <is>
+          <t>EXCLUDE</t>
+        </is>
+      </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="H53" s="3" t="inlineStr"/>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="H53" s="3" t="inlineStr">
+        <is>
+          <t>Ecological pollution nonlinear diffusion; physical, off-topic.</t>
+        </is>
+      </c>
       <c r="I53" s="3" t="inlineStr">
         <is>
-          <t>Quantum Fourier generative models; unclear if diffusion-based. Needs full text.</t>
+          <t>Ecological pollution nonlinear diffusion; physical, off-topic.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>2604.01197</t>
+          <t>2605.13268</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr"/>
@@ -2688,46 +2724,50 @@
       </c>
       <c r="D54" s="3" t="inlineStr">
         <is>
-          <t>Learning and Generating Mixed States Prepared by Shallow Channel Circuits</t>
+          <t>Physics Guided Generative Optimization for Trotter Suzuki Decomposition</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>CORE</t>
-        </is>
-      </c>
-      <c r="F54" s="6" t="inlineStr">
-        <is>
-          <t>MANUAL_REVIEW</t>
+          <t>RELATED</t>
+        </is>
+      </c>
+      <c r="F54" s="7" t="inlineStr">
+        <is>
+          <t>EXCLUDE</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="H54" s="3" t="inlineStr"/>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="H54" s="3" t="inlineStr">
+        <is>
+          <t>Removed in manual audit: insufficient relation to quantum diffusion models.</t>
+        </is>
+      </c>
       <c r="I54" s="3" t="inlineStr">
         <is>
-          <t>Generating mixed states via shallow channels; verify it is diffusion-based.</t>
+          <t>Reclassified from CORE/RELATED to EXCLUDE during manual audit (2026-07-13).</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>2310.07797</t>
+          <t>2501.05666</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr"/>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="D55" s="3" t="inlineStr">
         <is>
-          <t>Quantum sequential scattering model for quantum state learning</t>
+          <t>Diffusion-Enhanced Optimization of Variational Quantum Eigensolver for General Hamiltonians</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
@@ -2735,42 +2775,42 @@
           <t>CORE</t>
         </is>
       </c>
-      <c r="F55" s="6" t="inlineStr">
-        <is>
-          <t>MANUAL_REVIEW</t>
+      <c r="F55" s="7" t="inlineStr">
+        <is>
+          <t>EXCLUDE</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="H55" s="3" t="inlineStr"/>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="H55" s="3" t="inlineStr">
+        <is>
+          <t>Removed in manual audit: insufficient relation to quantum diffusion models.</t>
+        </is>
+      </c>
       <c r="I55" s="3" t="inlineStr">
         <is>
-          <t>Quantum sequential scattering for state learning; verify diffusion link.</t>
+          <t>Reclassified from CORE/RELATED to EXCLUDE during manual audit (2026-07-13).</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>2603.02834</t>
-        </is>
-      </c>
-      <c r="B56" s="2" t="inlineStr">
-        <is>
-          <t>10.15302/frontphys.2026.113201</t>
-        </is>
-      </c>
+          <t>2506.21015</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr"/>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="D56" s="3" t="inlineStr">
         <is>
-          <t>Identification of quantum generative circuits with parallel quantum neural network</t>
+          <t>MediQ-GAN: Quantum-Inspired GAN for High Resolution Medical Image Generation</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
@@ -2790,30 +2830,30 @@
       </c>
       <c r="H56" s="3" t="inlineStr">
         <is>
-          <t>Discriminative circuit identification (ParaQuanNet); not generative diffusion.</t>
+          <t>Quantum-inspired GAN, not a diffusion model.</t>
         </is>
       </c>
       <c r="I56" s="3" t="inlineStr">
         <is>
-          <t>Discriminative circuit identification (ParaQuanNet); not generative diffusion.</t>
+          <t>Quantum-inspired GAN, not a diffusion model.</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>2605.19754</t>
+          <t>2503.02345</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr"/>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="D57" s="3" t="inlineStr">
         <is>
-          <t>Hypothesis Tests for Observing Quantum Entanglement in HWW at the LHC</t>
+          <t>CQ CNN: A Hybrid Classical Quantum Convolutional Neural Network for Alzheimer's Disease Detection Using Diffusion Generated and U Net Segmented 3D MRI</t>
         </is>
       </c>
       <c r="E57" s="2" t="inlineStr">
@@ -2833,30 +2873,34 @@
       </c>
       <c r="H57" s="3" t="inlineStr">
         <is>
-          <t>LHC particle-physics entanglement hypothesis test; off-topic.</t>
+          <t>Hybrid classical-quantum CNN classifier; not diffusion.</t>
         </is>
       </c>
       <c r="I57" s="3" t="inlineStr">
         <is>
-          <t>LHC particle-physics entanglement hypothesis test; off-topic.</t>
+          <t>Hybrid classical-quantum CNN classifier; not diffusion.</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>2607.00566</t>
-        </is>
-      </c>
-      <c r="B58" s="2" t="inlineStr"/>
+          <t>2506.22755</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>10.1103/7717-1mw2</t>
+        </is>
+      </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="D58" s="3" t="inlineStr">
         <is>
-          <t>Effective Color Dipole Approach to Color Transparency in $ρ^0$ Electroproduction</t>
+          <t>Scaling Laws of Quantum Information Lifetime in Monitored Quantum Dynamics</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
@@ -2876,171 +2920,175 @@
       </c>
       <c r="H58" s="3" t="inlineStr">
         <is>
-          <t>Nuclear-physics color transparency; transport, not generative.</t>
+          <t>Monitored-dynamics physics; not a generative diffusion model.</t>
         </is>
       </c>
       <c r="I58" s="3" t="inlineStr">
         <is>
-          <t>Nuclear-physics color transparency; transport, not generative.</t>
+          <t>Monitored-dynamics physics; not a generative diffusion model.</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>2604.05612</t>
-        </is>
-      </c>
-      <c r="B59" s="2" t="inlineStr"/>
+          <t>2506.15331</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>10.1088/1674-1137/ae6b20</t>
+        </is>
+      </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="D59" s="3" t="inlineStr">
         <is>
-          <t>Deuteron normalization and channel-dependent formation dynamics in pion and kaon color transparency</t>
+          <t>Naive parton picture for kaon color transparency in $A(e,e'K^+)$</t>
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="F59" s="7" t="inlineStr">
+        <is>
+          <t>EXCLUDE</t>
+        </is>
+      </c>
+      <c r="G59" s="2" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="H59" s="3" t="inlineStr">
+        <is>
+          <t>Nuclear-physics kaon color transparency; off-topic.</t>
+        </is>
+      </c>
+      <c r="I59" s="3" t="inlineStr">
+        <is>
+          <t>Nuclear-physics kaon color transparency; off-topic.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>2512.19877</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr"/>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D60" s="3" t="inlineStr">
+        <is>
+          <t>Spectral Diffusion for Sampling on ${\rm SU}(N)$</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="inlineStr">
+        <is>
           <t>MANUAL_REVIEW</t>
         </is>
       </c>
-      <c r="F59" s="7" t="inlineStr">
+      <c r="F60" s="7" t="inlineStr">
         <is>
           <t>EXCLUDE</t>
         </is>
       </c>
-      <c r="G59" s="2" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="H59" s="3" t="inlineStr">
-        <is>
-          <t>Nuclear-physics color transparency; off-topic.</t>
-        </is>
-      </c>
-      <c r="I59" s="3" t="inlineStr">
-        <is>
-          <t>Nuclear-physics color transparency; off-topic.</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="2" t="inlineStr"/>
-      <c r="B60" s="2" t="inlineStr">
-        <is>
-          <t>10.1007/978-3-032-09973-0_7</t>
-        </is>
-      </c>
-      <c r="C60" s="2" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="D60" s="3" t="inlineStr">
-        <is>
-          <t>Ecological Pollution Control Using a Nonlinear Diffusion Model Based on Quantum Optimization</t>
-        </is>
-      </c>
-      <c r="E60" s="2" t="inlineStr">
+      <c r="G60" s="2" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="H60" s="3" t="inlineStr">
+        <is>
+          <t>Removed in manual audit: insufficient relation to quantum diffusion models.</t>
+        </is>
+      </c>
+      <c r="I60" s="3" t="inlineStr">
+        <is>
+          <t>Reclassified from CORE/RELATED to EXCLUDE during manual audit (2026-07-13).</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr"/>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>10.1109/sispad66650.2025.11185919</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D61" s="3" t="inlineStr">
+        <is>
+          <t>Discretization Methods for Quantum Drift-Diffusion Model: A Comparison Based on the Quasi-Fermi Scheme</t>
+        </is>
+      </c>
+      <c r="E61" s="2" t="inlineStr">
         <is>
           <t>MANUAL_REVIEW</t>
         </is>
       </c>
-      <c r="F60" s="7" t="inlineStr">
+      <c r="F61" s="7" t="inlineStr">
         <is>
           <t>EXCLUDE</t>
         </is>
       </c>
-      <c r="G60" s="2" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="H60" s="3" t="inlineStr">
-        <is>
-          <t>Ecological pollution nonlinear diffusion; physical, off-topic.</t>
-        </is>
-      </c>
-      <c r="I60" s="3" t="inlineStr">
-        <is>
-          <t>Ecological pollution nonlinear diffusion; physical, off-topic.</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="2" t="inlineStr">
-        <is>
-          <t>2506.21015</t>
-        </is>
-      </c>
-      <c r="B61" s="2" t="inlineStr"/>
-      <c r="C61" s="2" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="D61" s="3" t="inlineStr">
-        <is>
-          <t>MediQ-GAN: Quantum-Inspired GAN for High Resolution Medical Image Generation</t>
-        </is>
-      </c>
-      <c r="E61" s="2" t="inlineStr">
-        <is>
-          <t>CORE</t>
-        </is>
-      </c>
-      <c r="F61" s="7" t="inlineStr">
+      <c r="G61" s="2" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="H61" s="3" t="inlineStr">
+        <is>
+          <t>Semiconductor quantum drift-diffusion; physical transport, off-topic.</t>
+        </is>
+      </c>
+      <c r="I61" s="3" t="inlineStr">
+        <is>
+          <t>Semiconductor quantum drift-diffusion; physical transport, off-topic.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr"/>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>10.1109/qce60285.2024.10259</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="D62" s="3" t="inlineStr">
+        <is>
+          <t>QRNG-DDPM: Enhancing Diffusion Models Through Fitting Mixture Noise with Quantum Random Number</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="F62" s="7" t="inlineStr">
         <is>
           <t>EXCLUDE</t>
         </is>
       </c>
-      <c r="G61" s="2" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="H61" s="3" t="inlineStr">
-        <is>
-          <t>Quantum-inspired GAN, not a diffusion model.</t>
-        </is>
-      </c>
-      <c r="I61" s="3" t="inlineStr">
-        <is>
-          <t>Quantum-inspired GAN, not a diffusion model.</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="2" t="inlineStr">
-        <is>
-          <t>2503.02345</t>
-        </is>
-      </c>
-      <c r="B62" s="2" t="inlineStr"/>
-      <c r="C62" s="2" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="D62" s="3" t="inlineStr">
-        <is>
-          <t>CQ CNN: A Hybrid Classical Quantum Convolutional Neural Network for Alzheimer's Disease Detection Using Diffusion Generated and U Net Segmented 3D MRI</t>
-        </is>
-      </c>
-      <c r="E62" s="2" t="inlineStr">
-        <is>
-          <t>CORE</t>
-        </is>
-      </c>
-      <c r="F62" s="7" t="inlineStr">
-        <is>
-          <t>EXCLUDE</t>
-        </is>
-      </c>
       <c r="G62" s="2" t="inlineStr">
         <is>
           <t>high</t>
@@ -3048,34 +3096,30 @@
       </c>
       <c r="H62" s="3" t="inlineStr">
         <is>
-          <t>Hybrid classical-quantum CNN classifier; not diffusion.</t>
+          <t>Removed in manual audit: insufficient relation to quantum diffusion models.</t>
         </is>
       </c>
       <c r="I62" s="3" t="inlineStr">
         <is>
-          <t>Hybrid classical-quantum CNN classifier; not diffusion.</t>
+          <t>Reclassified from CORE/RELATED to EXCLUDE during manual audit (2026-07-13).</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>2506.22755</t>
-        </is>
-      </c>
-      <c r="B63" s="2" t="inlineStr">
-        <is>
-          <t>10.1103/7717-1mw2</t>
-        </is>
-      </c>
+          <t>2406.00503</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr"/>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="D63" s="3" t="inlineStr">
         <is>
-          <t>Scaling Laws of Quantum Information Lifetime in Monitored Quantum Dynamics</t>
+          <t>Schrödinger Bridge with Quadratic State Cost is Exactly Solvable</t>
         </is>
       </c>
       <c r="E63" s="2" t="inlineStr">
@@ -3090,39 +3134,35 @@
       </c>
       <c r="G63" s="2" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="H63" s="3" t="inlineStr">
         <is>
-          <t>Monitored-dynamics physics; not a generative diffusion model.</t>
+          <t>Classical Schrodinger-bridge control theory; not a quantum diffusion model.</t>
         </is>
       </c>
       <c r="I63" s="3" t="inlineStr">
         <is>
-          <t>Monitored-dynamics physics; not a generative diffusion model.</t>
+          <t>Classical Schrodinger-bridge control theory; not a quantum diffusion model.</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>2506.15331</t>
-        </is>
-      </c>
-      <c r="B64" s="2" t="inlineStr">
-        <is>
-          <t>10.1088/1674-1137/ae6b20</t>
-        </is>
-      </c>
+          <t>2409.05129</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr"/>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="D64" s="3" t="inlineStr">
         <is>
-          <t>Naive parton picture for kaon color transparency in $A(e,e'K^+)$</t>
+          <t>Nuclear transparency and shadowing of the two-step process in the $A(e,e'π^+)$ reaction</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
@@ -3142,12 +3182,12 @@
       </c>
       <c r="H64" s="3" t="inlineStr">
         <is>
-          <t>Nuclear-physics kaon color transparency; off-topic.</t>
+          <t>Nuclear transparency (Glauber); off-topic.</t>
         </is>
       </c>
       <c r="I64" s="3" t="inlineStr">
         <is>
-          <t>Nuclear-physics kaon color transparency; off-topic.</t>
+          <t>Nuclear transparency (Glauber); off-topic.</t>
         </is>
       </c>
     </row>
@@ -3155,17 +3195,17 @@
       <c r="A65" s="2" t="inlineStr"/>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>10.1109/sispad66650.2025.11185919</t>
+          <t>10.1109/ccpqt64497.2024.00016</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="D65" s="3" t="inlineStr">
         <is>
-          <t>Discretization Methods for Quantum Drift-Diffusion Model: A Comparison Based on the Quasi-Fermi Scheme</t>
+          <t>Adversarial Attacks Defense for Continuous Variable Quantum Key Distribution System Based on Diffusion Model</t>
         </is>
       </c>
       <c r="E65" s="2" t="inlineStr">
@@ -3185,22 +3225,22 @@
       </c>
       <c r="H65" s="3" t="inlineStr">
         <is>
-          <t>Semiconductor quantum drift-diffusion; physical transport, off-topic.</t>
+          <t>CV-QKD adversarial defense; not a generative diffusion model.</t>
         </is>
       </c>
       <c r="I65" s="3" t="inlineStr">
         <is>
-          <t>Semiconductor quantum drift-diffusion; physical transport, off-topic.</t>
+          <t>CV-QKD adversarial defense; not a generative diffusion model.</t>
         </is>
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="2" t="inlineStr">
-        <is>
-          <t>2406.00503</t>
-        </is>
-      </c>
-      <c r="B66" s="2" t="inlineStr"/>
+      <c r="A66" s="2" t="inlineStr"/>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>10.1007/jhep05(2024)060</t>
+        </is>
+      </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
           <t>2024</t>
@@ -3208,12 +3248,12 @@
       </c>
       <c r="D66" s="3" t="inlineStr">
         <is>
-          <t>Schrödinger Bridge with Quadratic State Cost is Exactly Solvable</t>
+          <t>Diffusion models as stochastic quantization in lattice field theory</t>
         </is>
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>CORE</t>
+          <t>MANUAL_REVIEW</t>
         </is>
       </c>
       <c r="F66" s="7" t="inlineStr">
@@ -3223,27 +3263,27 @@
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="H66" s="3" t="inlineStr">
         <is>
-          <t>Classical Schrodinger-bridge control theory; not a quantum diffusion model.</t>
+          <t>Removed in manual audit: insufficient relation to quantum diffusion models.</t>
         </is>
       </c>
       <c r="I66" s="3" t="inlineStr">
         <is>
-          <t>Classical Schrodinger-bridge control theory; not a quantum diffusion model.</t>
+          <t>Reclassified from CORE/RELATED to EXCLUDE during manual audit (2026-07-13).</t>
         </is>
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="2" t="inlineStr">
-        <is>
-          <t>2409.05129</t>
-        </is>
-      </c>
-      <c r="B67" s="2" t="inlineStr"/>
+      <c r="A67" s="2" t="inlineStr"/>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>10.1109/tpami.2024.3430839</t>
+        </is>
+      </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
           <t>2024</t>
@@ -3251,12 +3291,12 @@
       </c>
       <c r="D67" s="3" t="inlineStr">
         <is>
-          <t>Nuclear transparency and shadowing of the two-step process in the $A(e,e'π^+)$ reaction</t>
+          <t>STQD-Det: Spatio-Temporal Quantum Diffusion Model for Real-Time Coronary Stenosis Detection in X-Ray Angiography</t>
         </is>
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>CORE</t>
+          <t>MANUAL_REVIEW</t>
         </is>
       </c>
       <c r="F67" s="7" t="inlineStr">
@@ -3271,12 +3311,12 @@
       </c>
       <c r="H67" s="3" t="inlineStr">
         <is>
-          <t>Nuclear transparency (Glauber); off-topic.</t>
+          <t>Removed in manual audit: insufficient relation to quantum diffusion models.</t>
         </is>
       </c>
       <c r="I67" s="3" t="inlineStr">
         <is>
-          <t>Nuclear transparency (Glauber); off-topic.</t>
+          <t>Reclassified from CORE/RELATED to EXCLUDE during manual audit (2026-07-13).</t>
         </is>
       </c>
     </row>
@@ -3284,7 +3324,7 @@
       <c r="A68" s="2" t="inlineStr"/>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>10.1109/ccpqt64497.2024.00016</t>
+          <t>10.1109/iemcon62851.2024.11093551</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
@@ -3294,7 +3334,7 @@
       </c>
       <c r="D68" s="3" t="inlineStr">
         <is>
-          <t>Adversarial Attacks Defense for Continuous Variable Quantum Key Distribution System Based on Diffusion Model</t>
+          <t>A Latency Score based Benchmarking Framework integrating Quantum Computing in Edge-Cloud Environments</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr">
@@ -3314,35 +3354,35 @@
       </c>
       <c r="H68" s="3" t="inlineStr">
         <is>
-          <t>CV-QKD adversarial defense; not a generative diffusion model.</t>
+          <t>Latency-score benchmarking framework; not a QDM.</t>
         </is>
       </c>
       <c r="I68" s="3" t="inlineStr">
         <is>
-          <t>CV-QKD adversarial defense; not a generative diffusion model.</t>
+          <t>Latency-score benchmarking framework; not a QDM.</t>
         </is>
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="2" t="inlineStr"/>
-      <c r="B69" s="2" t="inlineStr">
-        <is>
-          <t>10.1109/iemcon62851.2024.11093551</t>
-        </is>
-      </c>
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>2305.16540</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="inlineStr"/>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2023</t>
         </is>
       </c>
       <c r="D69" s="3" t="inlineStr">
         <is>
-          <t>A Latency Score based Benchmarking Framework integrating Quantum Computing in Edge-Cloud Environments</t>
+          <t>A Score-Based Model for Learning Neural Wavefunctions</t>
         </is>
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>MANUAL_REVIEW</t>
+          <t>CORE</t>
         </is>
       </c>
       <c r="F69" s="7" t="inlineStr">
@@ -3357,12 +3397,12 @@
       </c>
       <c r="H69" s="3" t="inlineStr">
         <is>
-          <t>Latency-score benchmarking framework; not a QDM.</t>
+          <t>Removed in manual audit: insufficient relation to quantum diffusion models.</t>
         </is>
       </c>
       <c r="I69" s="3" t="inlineStr">
         <is>
-          <t>Latency-score benchmarking framework; not a QDM.</t>
+          <t>Reclassified from CORE/RELATED to EXCLUDE during manual audit (2026-07-13).</t>
         </is>
       </c>
     </row>
@@ -3558,17 +3598,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="52" customWidth="1" min="1" max="1"/>
+    <col width="54" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="8" t="inlineStr">
         <is>
-          <t>Screening summary — full field, all years (2020–2026)</t>
+          <t>Screening summary — full field, all years (2020–2026), audited 2026-07-13</t>
         </is>
       </c>
     </row>
@@ -3591,7 +3631,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>48</v>
+        <v>40</v>
       </c>
     </row>
     <row r="5">
@@ -3601,7 +3641,7 @@
         </is>
       </c>
       <c r="B5" s="10" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6">
@@ -3621,7 +3661,7 @@
         </is>
       </c>
       <c r="B7" s="10" t="n">
-        <v>18</v>
+        <v>28</v>
       </c>
     </row>
     <row r="8">
@@ -3634,17 +3674,10 @@
         <v>72</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="8" t="inlineStr">
-        <is>
-          <t>CORE = review corpus (primary quantum diffusion studies). RELATED = supporting (e.g. metrics, GAN, non-diffusion). MANUAL_REVIEW = needs full-text. EXCLUDE = physical diffusion / off-topic false positives.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="8" t="inlineStr">
-        <is>
-          <t>Built from the automated shortlist: papers_core (54) + papers_manual_review (17) + papers_related (1) = 72 records, human-screened.</t>
+    <row r="10">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>CORE = review corpus (primary quantum diffusion studies). Audited manually: 10 records reclassified CORE/RELATED -&gt; EXCLUDE.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Consolidate few-shot duplicate: review corpus now 39 CORE; regenerate screening flow, PRISMA and tests
</commit_message>
<xml_diff>
--- a/data/screening/manual_screening.xlsx
+++ b/data/screening/manual_screening.xlsx
@@ -1071,25 +1071,25 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="inlineStr"/>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>10.1007/978-3-032-15931-1_4</t>
-        </is>
-      </c>
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>2512.06695</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr"/>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>Quantum Diffusion Models for Few-Shot Learning</t>
+          <t>Mitigating Barren Plateaus in Quantum Denoising Diffusion Probabilistic Model</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>MANUAL_REVIEW</t>
+          <t>CORE</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
@@ -1099,20 +1099,20 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="H14" s="3" t="inlineStr"/>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>QDM for few-shot learning (book chapter; possible duplicate of 2411.04217).</t>
+          <t>QuDDPM barren-plateau mitigation.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>2512.06695</t>
+          <t>2505.05151</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr"/>
@@ -1123,7 +1123,7 @@
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>Mitigating Barren Plateaus in Quantum Denoising Diffusion Probabilistic Model</t>
+          <t>Overcoming Dimensional Factorization Limits in Discrete Diffusion Models through Quantum Joint Distribution Learning</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
@@ -1144,14 +1144,14 @@
       <c r="H15" s="3" t="inlineStr"/>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>QuDDPM barren-plateau mitigation.</t>
+          <t>Quantum discrete diffusion (dimensional factorization limits).</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2505.05151</t>
+          <t>2509.17569</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr"/>
@@ -1162,7 +1162,7 @@
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>Overcoming Dimensional Factorization Limits in Discrete Diffusion Models through Quantum Joint Distribution Learning</t>
+          <t>Conditioning in Generative Quantum Denoising Diffusion Models</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
@@ -1183,17 +1183,21 @@
       <c r="H16" s="3" t="inlineStr"/>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>Quantum discrete diffusion (dimensional factorization limits).</t>
+          <t>Conditioning in generative QuDDPM.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>2509.17569</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="inlineStr"/>
+          <t>2506.01666</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>10.1088/2632-2153/ae5b21</t>
+        </is>
+      </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
           <t>2025</t>
@@ -1201,7 +1205,7 @@
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>Conditioning in Generative Quantum Denoising Diffusion Models</t>
+          <t>Synthesis of discrete-continuous quantum circuits with multimodal diffusion models</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
@@ -1222,21 +1226,17 @@
       <c r="H17" s="3" t="inlineStr"/>
       <c r="I17" s="3" t="inlineStr">
         <is>
-          <t>Conditioning in generative QuDDPM.</t>
+          <t>Multimodal diffusion for discrete-continuous circuit synthesis.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2506.01666</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>10.1088/2632-2153/ae5b21</t>
-        </is>
-      </c>
+          <t>2506.19270</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr"/>
       <c r="C18" s="2" t="inlineStr">
         <is>
           <t>2025</t>
@@ -1244,7 +1244,7 @@
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>Synthesis of discrete-continuous quantum circuits with multimodal diffusion models</t>
+          <t>Continuous-variable Quantum Diffusion Model for State Generation and Restoration</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
@@ -1265,14 +1265,14 @@
       <c r="H18" s="3" t="inlineStr"/>
       <c r="I18" s="3" t="inlineStr">
         <is>
-          <t>Multimodal diffusion for discrete-continuous circuit synthesis.</t>
+          <t>Continuous-variable quantum diffusion model.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>2506.19270</t>
+          <t>2501.16380</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr"/>
@@ -1283,7 +1283,7 @@
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>Continuous-variable Quantum Diffusion Model for State Generation and Restoration</t>
+          <t>UDiTQC: U-Net-Style Diffusion Transformer for Quantum Circuit Synthesis</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
@@ -1304,14 +1304,14 @@
       <c r="H19" s="3" t="inlineStr"/>
       <c r="I19" s="3" t="inlineStr">
         <is>
-          <t>Continuous-variable quantum diffusion model.</t>
+          <t>U-Net diffusion transformer for quantum circuit synthesis.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2501.16380</t>
+          <t>2505.22193</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr"/>
@@ -1322,7 +1322,7 @@
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>UDiTQC: U-Net-Style Diffusion Transformer for Quantum Circuit Synthesis</t>
+          <t>Physics-inspired Generative AI models via real hardware-based noisy quantum diffusion</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
@@ -1343,14 +1343,14 @@
       <c r="H20" s="3" t="inlineStr"/>
       <c r="I20" s="3" t="inlineStr">
         <is>
-          <t>U-Net diffusion transformer for quantum circuit synthesis.</t>
+          <t>Noise-driven QDM on real hardware.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>2505.22193</t>
+          <t>2508.08799</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr"/>
@@ -1361,7 +1361,7 @@
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>Physics-inspired Generative AI models via real hardware-based noisy quantum diffusion</t>
+          <t>Measurement-Based Quantum Diffusion Models</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
@@ -1382,17 +1382,21 @@
       <c r="H21" s="3" t="inlineStr"/>
       <c r="I21" s="3" t="inlineStr">
         <is>
-          <t>Noise-driven QDM on real hardware.</t>
+          <t>Measurement-based quantum diffusion.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2508.08799</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="inlineStr"/>
+          <t>2505.20863</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>10.1109/qce65121.2025.00180</t>
+        </is>
+      </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
           <t>2025</t>
@@ -1400,7 +1404,7 @@
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>Measurement-Based Quantum Diffusion Models</t>
+          <t>Leveraging Diffusion Models for Parameterized Quantum Circuit Generation</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
@@ -1421,21 +1425,17 @@
       <c r="H22" s="3" t="inlineStr"/>
       <c r="I22" s="3" t="inlineStr">
         <is>
-          <t>Measurement-based quantum diffusion.</t>
+          <t>Diffusion for parameterized quantum circuit generation (Barta).</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>2505.20863</t>
-        </is>
-      </c>
-      <c r="B23" s="2" t="inlineStr">
-        <is>
-          <t>10.1109/qce65121.2025.00180</t>
-        </is>
-      </c>
+          <t>2511.12221</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr"/>
       <c r="C23" s="2" t="inlineStr">
         <is>
           <t>2025</t>
@@ -1443,7 +1443,7 @@
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>Leveraging Diffusion Models for Parameterized Quantum Circuit Generation</t>
+          <t>Channel-Constrained Markovian Quantum Diffusion Model from Open System Perspective</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
@@ -1464,17 +1464,21 @@
       <c r="H23" s="3" t="inlineStr"/>
       <c r="I23" s="3" t="inlineStr">
         <is>
-          <t>Diffusion for parameterized quantum circuit generation (Barta).</t>
+          <t>Open-system Markovian quantum diffusion (CCMQD).</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2511.12221</t>
-        </is>
-      </c>
-      <c r="B24" s="2" t="inlineStr"/>
+          <t>2411.15973</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>10.1007/978-3-031-78395-1_23</t>
+        </is>
+      </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
           <t>2025</t>
@@ -1482,7 +1486,7 @@
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>Channel-Constrained Markovian Quantum Diffusion Model from Open System Perspective</t>
+          <t>Enhancing Quantum Diffusion Models with Pairwise Bell State Entanglement</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
@@ -1503,19 +1507,19 @@
       <c r="H24" s="3" t="inlineStr"/>
       <c r="I24" s="3" t="inlineStr">
         <is>
-          <t>Open-system Markovian quantum diffusion (CCMQD).</t>
+          <t>Bell-state entanglement QDM.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>2411.15973</t>
+          <t>2508.09903</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>10.1007/978-3-031-78395-1_23</t>
+          <t>10.1109/qce65121.2025.10364</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
@@ -1525,7 +1529,7 @@
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>Enhancing Quantum Diffusion Models with Pairwise Bell State Entanglement</t>
+          <t>Hybrid Quantum-Classical Latent Diffusion Models for Medical Image Generation</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
@@ -1546,19 +1550,19 @@
       <c r="H25" s="3" t="inlineStr"/>
       <c r="I25" s="3" t="inlineStr">
         <is>
-          <t>Bell-state entanglement QDM.</t>
+          <t>Hybrid latent QDM for medical imaging.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2508.09903</t>
+          <t>2411.04217</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>10.1109/qce65121.2025.10364</t>
+          <t>10.1109/icad65464.2025.11114033</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -1568,7 +1572,7 @@
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>Hybrid Quantum-Classical Latent Diffusion Models for Medical Image Generation</t>
+          <t>Quantum Diffusion Models for Few-Shot Learning</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
@@ -1589,19 +1593,19 @@
       <c r="H26" s="3" t="inlineStr"/>
       <c r="I26" s="3" t="inlineStr">
         <is>
-          <t>Hybrid latent QDM for medical imaging.</t>
+          <t>QDM for few-shot learning.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>2411.04217</t>
+          <t>2406.00843</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>10.1109/icad65464.2025.11114033</t>
+          <t>10.1007/s42484-025-00276-2</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
@@ -1611,7 +1615,7 @@
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>Quantum Diffusion Models for Few-Shot Learning</t>
+          <t>Diffusion-inspired quantum noise mitigation in parameterized quantum circuits</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
@@ -1626,25 +1630,25 @@
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="H27" s="3" t="inlineStr"/>
       <c r="I27" s="3" t="inlineStr">
         <is>
-          <t>QDM for few-shot learning.</t>
+          <t>Diffusion-inspired quantum noise mitigation in PQCs (QMI).</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2406.00843</t>
+          <t>2501.11174</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>10.1007/s42484-025-00276-2</t>
+          <t>10.1007/s42484-024-00224-6</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
@@ -1654,12 +1658,12 @@
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>Diffusion-inspired quantum noise mitigation in parameterized quantum circuits</t>
+          <t>Quantum Latent Diffusion Models</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>CORE</t>
+          <t>MANUAL_REVIEW</t>
         </is>
       </c>
       <c r="F28" s="4" t="inlineStr">
@@ -1669,25 +1673,21 @@
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="H28" s="3" t="inlineStr"/>
       <c r="I28" s="3" t="inlineStr">
         <is>
-          <t>Diffusion-inspired quantum noise mitigation in PQCs (QMI).</t>
+          <t>Quantum Latent Diffusion Models (De Falco, QMI).</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="2" t="inlineStr">
-        <is>
-          <t>2501.11174</t>
-        </is>
-      </c>
+      <c r="A29" s="2" t="inlineStr"/>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>10.1007/s42484-024-00224-6</t>
+          <t>10.1109/ijcnn64981.2025.11227283</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
@@ -1697,7 +1697,7 @@
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>Quantum Latent Diffusion Models</t>
+          <t>Hybrid and hardware-oriented approaches for quantum diffusion models</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
@@ -1718,7 +1718,7 @@
       <c r="H29" s="3" t="inlineStr"/>
       <c r="I29" s="3" t="inlineStr">
         <is>
-          <t>Quantum Latent Diffusion Models (De Falco, QMI).</t>
+          <t>Hybrid hardware-oriented quantum diffusion approaches.</t>
         </is>
       </c>
     </row>
@@ -1726,7 +1726,7 @@
       <c r="A30" s="2" t="inlineStr"/>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>10.1109/ijcnn64981.2025.11227283</t>
+          <t>10.1109/igarss55030.2025.11242723</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
@@ -1736,7 +1736,7 @@
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>Hybrid and hardware-oriented approaches for quantum diffusion models</t>
+          <t>Leveraging Quantum Latent Diffusion Models for Data Augmentation on The Eurosat Dataset</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
@@ -1757,30 +1757,30 @@
       <c r="H30" s="3" t="inlineStr"/>
       <c r="I30" s="3" t="inlineStr">
         <is>
-          <t>Hybrid hardware-oriented quantum diffusion approaches.</t>
+          <t>Quantum latent diffusion for EuroSAT data augmentation.</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="2" t="inlineStr"/>
-      <c r="B31" s="2" t="inlineStr">
-        <is>
-          <t>10.1109/igarss55030.2025.11242723</t>
-        </is>
-      </c>
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>2411.17608</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr"/>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>Leveraging Quantum Latent Diffusion Models for Data Augmentation on The Eurosat Dataset</t>
+          <t>Mixed-State Quantum Denoising Diffusion Probabilistic Model</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>MANUAL_REVIEW</t>
+          <t>CORE</t>
         </is>
       </c>
       <c r="F31" s="4" t="inlineStr">
@@ -1796,14 +1796,14 @@
       <c r="H31" s="3" t="inlineStr"/>
       <c r="I31" s="3" t="inlineStr">
         <is>
-          <t>Quantum latent diffusion for EuroSAT data augmentation.</t>
+          <t>Mixed-state QuDDPM (Kwun).</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2411.17608</t>
+          <t>2407.12242</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr"/>
@@ -1814,7 +1814,7 @@
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>Mixed-State Quantum Denoising Diffusion Probabilistic Model</t>
+          <t>Conditional Diffusion-based Parameter Generation for Quantum Approximate Optimization Algorithm</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
@@ -1835,17 +1835,21 @@
       <c r="H32" s="3" t="inlineStr"/>
       <c r="I32" s="3" t="inlineStr">
         <is>
-          <t>Mixed-state QuDDPM (Kwun).</t>
+          <t>Conditional diffusion for QAOA parameter generation.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>2407.12242</t>
-        </is>
-      </c>
-      <c r="B33" s="2" t="inlineStr"/>
+          <t>2401.07049</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>10.1109/qsw62656.2024.00023</t>
+        </is>
+      </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
           <t>2024</t>
@@ -1853,7 +1857,7 @@
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>Conditional Diffusion-based Parameter Generation for Quantum Approximate Optimization Algorithm</t>
+          <t>Quantum Denoising Diffusion Models</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
@@ -1874,21 +1878,17 @@
       <c r="H33" s="3" t="inlineStr"/>
       <c r="I33" s="3" t="inlineStr">
         <is>
-          <t>Conditional diffusion for QAOA parameter generation.</t>
+          <t>Quantum Denoising Diffusion Models (Kolle).</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2401.07049</t>
-        </is>
-      </c>
-      <c r="B34" s="2" t="inlineStr">
-        <is>
-          <t>10.1109/qsw62656.2024.00023</t>
-        </is>
-      </c>
+          <t>2412.21082</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr"/>
       <c r="C34" s="2" t="inlineStr">
         <is>
           <t>2024</t>
@@ -1896,7 +1896,7 @@
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>Quantum Denoising Diffusion Models</t>
+          <t>Quantum Diffusion Model for Quark and Gluon Jet Generation</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
@@ -1917,17 +1917,21 @@
       <c r="H34" s="3" t="inlineStr"/>
       <c r="I34" s="3" t="inlineStr">
         <is>
-          <t>Quantum Denoising Diffusion Models (Kolle).</t>
+          <t>QDM for quark/gluon jet generation.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>2412.21082</t>
-        </is>
-      </c>
-      <c r="B35" s="2" t="inlineStr"/>
+          <t>2402.16147</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>10.1007/s13218-024-00858-5</t>
+        </is>
+      </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
           <t>2024</t>
@@ -1935,7 +1939,7 @@
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>Quantum Diffusion Model for Quark and Gluon Jet Generation</t>
+          <t>Towards Efficient Quantum Hybrid Diffusion Models</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
@@ -1956,19 +1960,15 @@
       <c r="H35" s="3" t="inlineStr"/>
       <c r="I35" s="3" t="inlineStr">
         <is>
-          <t>QDM for quark/gluon jet generation.</t>
+          <t>Towards efficient quantum hybrid diffusion (De Falco).</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="2" t="inlineStr">
-        <is>
-          <t>2402.16147</t>
-        </is>
-      </c>
+      <c r="A36" s="2" t="inlineStr"/>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>10.1007/s13218-024-00858-5</t>
+          <t>10.1109/qce60285.2024.10371</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -1978,12 +1978,12 @@
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>Towards Efficient Quantum Hybrid Diffusion Models</t>
+          <t>Understanding of the Diffusion Noise in Quantum Latent Diffusion Model</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>CORE</t>
+          <t>MANUAL_REVIEW</t>
         </is>
       </c>
       <c r="F36" s="4" t="inlineStr">
@@ -1993,36 +1993,40 @@
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="H36" s="3" t="inlineStr"/>
       <c r="I36" s="3" t="inlineStr">
         <is>
-          <t>Towards efficient quantum hybrid diffusion (De Falco).</t>
+          <t>Analysis of diffusion noise in quantum latent diffusion.</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="2" t="inlineStr"/>
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>2311.02041</t>
+        </is>
+      </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>10.1109/qce60285.2024.10371</t>
+          <t>10.1038/s42256-024-00831-9</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2023</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>Understanding of the Diffusion Noise in Quantum Latent Diffusion Model</t>
+          <t>Quantum circuit synthesis with diffusion models</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>MANUAL_REVIEW</t>
+          <t>CORE</t>
         </is>
       </c>
       <c r="F37" s="4" t="inlineStr">
@@ -2032,27 +2036,23 @@
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="H37" s="3" t="inlineStr"/>
       <c r="I37" s="3" t="inlineStr">
         <is>
-          <t>Analysis of diffusion noise in quantum latent diffusion.</t>
+          <t>Quantum circuit synthesis with diffusion (genQC, Furrutter).</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2311.02041</t>
-        </is>
-      </c>
-      <c r="B38" s="2" t="inlineStr">
-        <is>
-          <t>10.1038/s42256-024-00831-9</t>
-        </is>
-      </c>
+          <t>2310.02511</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr"/>
       <c r="C38" s="2" t="inlineStr">
         <is>
           <t>2023</t>
@@ -2060,7 +2060,7 @@
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>Quantum circuit synthesis with diffusion models</t>
+          <t>Prepare Ansatz for VQE with Diffusion Model</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
@@ -2081,14 +2081,14 @@
       <c r="H38" s="3" t="inlineStr"/>
       <c r="I38" s="3" t="inlineStr">
         <is>
-          <t>Quantum circuit synthesis with diffusion (genQC, Furrutter).</t>
+          <t>Diffusion model to prepare VQE ansatz.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>2310.02511</t>
+          <t>2311.15444</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr"/>
@@ -2099,7 +2099,7 @@
       </c>
       <c r="D39" s="3" t="inlineStr">
         <is>
-          <t>Prepare Ansatz for VQE with Diffusion Model</t>
+          <t>Quantum Diffusion Models</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
@@ -2120,17 +2120,21 @@
       <c r="H39" s="3" t="inlineStr"/>
       <c r="I39" s="3" t="inlineStr">
         <is>
-          <t>Diffusion model to prepare VQE ansatz.</t>
+          <t>Quantum Diffusion Models (Cacioppo).</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2311.15444</t>
-        </is>
-      </c>
-      <c r="B40" s="2" t="inlineStr"/>
+          <t>2310.05866</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>10.1103/physrevlett.132.100602</t>
+        </is>
+      </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
           <t>2023</t>
@@ -2138,12 +2142,12 @@
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>Quantum Diffusion Models</t>
+          <t>Generative quantum machine learning via denoising diffusion probabilistic models</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>CORE</t>
+          <t>MANUAL_REVIEW</t>
         </is>
       </c>
       <c r="F40" s="4" t="inlineStr">
@@ -2159,39 +2163,35 @@
       <c r="H40" s="3" t="inlineStr"/>
       <c r="I40" s="3" t="inlineStr">
         <is>
-          <t>Quantum Diffusion Models (Cacioppo).</t>
+          <t>Generative QML via DDPM (Zhang QuDDPM; foundational).</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>2310.05866</t>
-        </is>
-      </c>
-      <c r="B41" s="2" t="inlineStr">
-        <is>
-          <t>10.1103/physrevlett.132.100602</t>
-        </is>
-      </c>
+          <t>2601.22005</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr"/>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>Generative quantum machine learning via denoising diffusion probabilistic models</t>
+          <t>Hierarchy of discriminative power and complexity in learning quantum ensembles</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>MANUAL_REVIEW</t>
-        </is>
-      </c>
-      <c r="F41" s="4" t="inlineStr">
-        <is>
-          <t>CORE</t>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="F41" s="5" t="inlineStr">
+        <is>
+          <t>RELATED</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
@@ -2202,14 +2202,14 @@
       <c r="H41" s="3" t="inlineStr"/>
       <c r="I41" s="3" t="inlineStr">
         <is>
-          <t>Generative QML via DDPM (Zhang QuDDPM; foundational).</t>
+          <t>MMD-k evaluation metric for quantum ensembles; supporting, not a generative model.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2601.22005</t>
+          <t>2606.28483</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr"/>
@@ -2220,7 +2220,7 @@
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t>Hierarchy of discriminative power and complexity in learning quantum ensembles</t>
+          <t>Quantum Fourier Generative Models Trainable at Large Scale</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
@@ -2228,27 +2228,27 @@
           <t>CORE</t>
         </is>
       </c>
-      <c r="F42" s="5" t="inlineStr">
-        <is>
-          <t>RELATED</t>
+      <c r="F42" s="6" t="inlineStr">
+        <is>
+          <t>MANUAL_REVIEW</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="H42" s="3" t="inlineStr"/>
       <c r="I42" s="3" t="inlineStr">
         <is>
-          <t>MMD-k evaluation metric for quantum ensembles; supporting, not a generative model.</t>
+          <t>Quantum Fourier generative models; unclear if diffusion-based. Needs full text.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>2606.28483</t>
+          <t>2604.01197</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr"/>
@@ -2259,7 +2259,7 @@
       </c>
       <c r="D43" s="3" t="inlineStr">
         <is>
-          <t>Quantum Fourier Generative Models Trainable at Large Scale</t>
+          <t>Learning and Generating Mixed States Prepared by Shallow Channel Circuits</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
@@ -2280,25 +2280,25 @@
       <c r="H43" s="3" t="inlineStr"/>
       <c r="I43" s="3" t="inlineStr">
         <is>
-          <t>Quantum Fourier generative models; unclear if diffusion-based. Needs full text.</t>
+          <t>Generating mixed states via shallow channels; verify it is diffusion-based.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2604.01197</t>
+          <t>2310.07797</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr"/>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2023</t>
         </is>
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>Learning and Generating Mixed States Prepared by Shallow Channel Circuits</t>
+          <t>Quantum sequential scattering model for quantum state learning</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
@@ -2319,25 +2319,29 @@
       <c r="H44" s="3" t="inlineStr"/>
       <c r="I44" s="3" t="inlineStr">
         <is>
-          <t>Generating mixed states via shallow channels; verify it is diffusion-based.</t>
+          <t>Quantum sequential scattering for state learning; verify diffusion link.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>2310.07797</t>
-        </is>
-      </c>
-      <c r="B45" s="2" t="inlineStr"/>
+          <t>2603.02834</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>10.15302/frontphys.2026.113201</t>
+        </is>
+      </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
         <is>
-          <t>Quantum sequential scattering model for quantum state learning</t>
+          <t>Identification of quantum generative circuits with parallel quantum neural network</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
@@ -2345,34 +2349,34 @@
           <t>CORE</t>
         </is>
       </c>
-      <c r="F45" s="6" t="inlineStr">
-        <is>
-          <t>MANUAL_REVIEW</t>
+      <c r="F45" s="7" t="inlineStr">
+        <is>
+          <t>EXCLUDE</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="H45" s="3" t="inlineStr"/>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="H45" s="3" t="inlineStr">
+        <is>
+          <t>Discriminative circuit identification (ParaQuanNet); not generative diffusion.</t>
+        </is>
+      </c>
       <c r="I45" s="3" t="inlineStr">
         <is>
-          <t>Quantum sequential scattering for state learning; verify diffusion link.</t>
+          <t>Discriminative circuit identification (ParaQuanNet); not generative diffusion.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2603.02834</t>
-        </is>
-      </c>
-      <c r="B46" s="2" t="inlineStr">
-        <is>
-          <t>10.15302/frontphys.2026.113201</t>
-        </is>
-      </c>
+          <t>2604.21210</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr"/>
       <c r="C46" s="2" t="inlineStr">
         <is>
           <t>2026</t>
@@ -2380,7 +2384,7 @@
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t>Identification of quantum generative circuits with parallel quantum neural network</t>
+          <t>The Feedback Hamiltonian is the Score Function: A Diffusion-Model Framework for Quantum Trajectory Reversal</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
@@ -2400,19 +2404,19 @@
       </c>
       <c r="H46" s="3" t="inlineStr">
         <is>
-          <t>Discriminative circuit identification (ParaQuanNet); not generative diffusion.</t>
+          <t>Removed in manual audit: insufficient relation to quantum diffusion models.</t>
         </is>
       </c>
       <c r="I46" s="3" t="inlineStr">
         <is>
-          <t>Discriminative circuit identification (ParaQuanNet); not generative diffusion.</t>
+          <t>Reclassified from CORE/RELATED to EXCLUDE during manual audit (2026-07-13).</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>2604.21210</t>
+          <t>2605.19754</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr"/>
@@ -2423,7 +2427,7 @@
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t>The Feedback Hamiltonian is the Score Function: A Diffusion-Model Framework for Quantum Trajectory Reversal</t>
+          <t>Hypothesis Tests for Observing Quantum Entanglement in HWW at the LHC</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
@@ -2443,19 +2447,19 @@
       </c>
       <c r="H47" s="3" t="inlineStr">
         <is>
-          <t>Removed in manual audit: insufficient relation to quantum diffusion models.</t>
+          <t>LHC particle-physics entanglement hypothesis test; off-topic.</t>
         </is>
       </c>
       <c r="I47" s="3" t="inlineStr">
         <is>
-          <t>Reclassified from CORE/RELATED to EXCLUDE during manual audit (2026-07-13).</t>
+          <t>LHC particle-physics entanglement hypothesis test; off-topic.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2605.19754</t>
+          <t>2605.23403</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr"/>
@@ -2466,7 +2470,7 @@
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>Hypothesis Tests for Observing Quantum Entanglement in HWW at the LHC</t>
+          <t>Hybrid Quantum-Classical Corrective Diffusion Modeling for Meteorological Downscaling</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
@@ -2486,19 +2490,19 @@
       </c>
       <c r="H48" s="3" t="inlineStr">
         <is>
-          <t>LHC particle-physics entanglement hypothesis test; off-topic.</t>
+          <t>Removed in manual audit: insufficient relation to quantum diffusion models.</t>
         </is>
       </c>
       <c r="I48" s="3" t="inlineStr">
         <is>
-          <t>LHC particle-physics entanglement hypothesis test; off-topic.</t>
+          <t>Reclassified from CORE/RELATED to EXCLUDE during manual audit (2026-07-13).</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>2605.23403</t>
+          <t>2606.05217</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr"/>
@@ -2509,7 +2513,7 @@
       </c>
       <c r="D49" s="3" t="inlineStr">
         <is>
-          <t>Hybrid Quantum-Classical Corrective Diffusion Modeling for Meteorological Downscaling</t>
+          <t>The Score Hamiltonian: Mapping Diffusion Models to Adiabatic Transport</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
@@ -2541,7 +2545,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2606.05217</t>
+          <t>2607.00566</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr"/>
@@ -2552,7 +2556,7 @@
       </c>
       <c r="D50" s="3" t="inlineStr">
         <is>
-          <t>The Score Hamiltonian: Mapping Diffusion Models to Adiabatic Transport</t>
+          <t>Effective Color Dipole Approach to Color Transparency in $ρ^0$ Electroproduction</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
@@ -2572,19 +2576,19 @@
       </c>
       <c r="H50" s="3" t="inlineStr">
         <is>
-          <t>Removed in manual audit: insufficient relation to quantum diffusion models.</t>
+          <t>Nuclear-physics color transparency; transport, not generative.</t>
         </is>
       </c>
       <c r="I50" s="3" t="inlineStr">
         <is>
-          <t>Reclassified from CORE/RELATED to EXCLUDE during manual audit (2026-07-13).</t>
+          <t>Nuclear-physics color transparency; transport, not generative.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>2607.00566</t>
+          <t>2604.05612</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr"/>
@@ -2595,12 +2599,12 @@
       </c>
       <c r="D51" s="3" t="inlineStr">
         <is>
-          <t>Effective Color Dipole Approach to Color Transparency in $ρ^0$ Electroproduction</t>
+          <t>Deuteron normalization and channel-dependent formation dynamics in pion and kaon color transparency</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>CORE</t>
+          <t>MANUAL_REVIEW</t>
         </is>
       </c>
       <c r="F51" s="7" t="inlineStr">
@@ -2615,22 +2619,22 @@
       </c>
       <c r="H51" s="3" t="inlineStr">
         <is>
-          <t>Nuclear-physics color transparency; transport, not generative.</t>
+          <t>Nuclear-physics color transparency; off-topic.</t>
         </is>
       </c>
       <c r="I51" s="3" t="inlineStr">
         <is>
-          <t>Nuclear-physics color transparency; transport, not generative.</t>
+          <t>Nuclear-physics color transparency; off-topic.</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="2" t="inlineStr">
-        <is>
-          <t>2604.05612</t>
-        </is>
-      </c>
-      <c r="B52" s="2" t="inlineStr"/>
+      <c r="A52" s="2" t="inlineStr"/>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>10.1007/978-3-032-09973-0_7</t>
+        </is>
+      </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
           <t>2026</t>
@@ -2638,7 +2642,7 @@
       </c>
       <c r="D52" s="3" t="inlineStr">
         <is>
-          <t>Deuteron normalization and channel-dependent formation dynamics in pion and kaon color transparency</t>
+          <t>Ecological Pollution Control Using a Nonlinear Diffusion Model Based on Quantum Optimization</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
@@ -2658,12 +2662,12 @@
       </c>
       <c r="H52" s="3" t="inlineStr">
         <is>
-          <t>Nuclear-physics color transparency; off-topic.</t>
+          <t>Ecological pollution nonlinear diffusion; physical, off-topic.</t>
         </is>
       </c>
       <c r="I52" s="3" t="inlineStr">
         <is>
-          <t>Nuclear-physics color transparency; off-topic.</t>
+          <t>Ecological pollution nonlinear diffusion; physical, off-topic.</t>
         </is>
       </c>
     </row>
@@ -2671,7 +2675,7 @@
       <c r="A53" s="2" t="inlineStr"/>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>10.1007/978-3-032-09973-0_7</t>
+          <t>10.1007/978-3-032-15931-1_4</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
@@ -2681,7 +2685,7 @@
       </c>
       <c r="D53" s="3" t="inlineStr">
         <is>
-          <t>Ecological Pollution Control Using a Nonlinear Diffusion Model Based on Quantum Optimization</t>
+          <t>Quantum Diffusion Models for Few-Shot Learning</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
@@ -2701,12 +2705,12 @@
       </c>
       <c r="H53" s="3" t="inlineStr">
         <is>
-          <t>Ecological pollution nonlinear diffusion; physical, off-topic.</t>
+          <t>Duplicate of arXiv:2411.04217 (same few-shot learning study); consolidated during manual deduplication.</t>
         </is>
       </c>
       <c r="I53" s="3" t="inlineStr">
         <is>
-          <t>Ecological pollution nonlinear diffusion; physical, off-topic.</t>
+          <t>Book-chapter version of 2411.04217; removed as duplicate (2026-07-13).</t>
         </is>
       </c>
     </row>
@@ -3601,14 +3605,14 @@
   <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="54" customWidth="1" min="1" max="1"/>
+    <col width="56" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="8" t="inlineStr">
         <is>
-          <t>Screening summary — full field, all years (2020–2026), audited 2026-07-13</t>
+          <t>Screening summary — full field, all years, audited 2026-07-13</t>
         </is>
       </c>
     </row>
@@ -3631,7 +3635,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="5">
@@ -3661,7 +3665,7 @@
         </is>
       </c>
       <c r="B7" s="10" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="8">
@@ -3677,7 +3681,7 @@
     <row r="10">
       <c r="A10" s="8" t="inlineStr">
         <is>
-          <t>CORE = review corpus (primary quantum diffusion studies). Audited manually: 10 records reclassified CORE/RELATED -&gt; EXCLUDE.</t>
+          <t>CORE = review corpus (39). Audited: 10 records CORE/RELATED-&gt;EXCLUDE + 1 few-shot duplicate consolidated.</t>
         </is>
       </c>
     </row>

</xml_diff>